<commit_message>
Corregir Freezing Points según MPP PG-001 Rev A — 09-JUN-2026
Correcciones críticas detectadas al comparar Excel vs MPP real:
- FP-S3-3 "Último FP ABB": 31-AGO-2026 → 26-OCT-2026 (+56d)
- FP-S4-3 / Sala 4 ID:     28-AGO-2026 → 06-OCT-2026 (+39d)
- FP-S3-2 / Sala 3 ID:     14-AGO-2026 → 06-OCT-2026 (+53d)
- FP-S4-1 / Sala 4 IB building: 26-JUN → 21-JUL (+25d)
- FP-S3-1 / Sala 3 IB building: 03-JUL → 21-JUL (+18d)
Sheet 4 reconstruida con 20 FPs del MPP (11 nuevos por equipo) + tabla comparativa

https://claude.ai/code/session_017wF27KL2NtMGeTJBXCBM3L
</commit_message>
<xml_diff>
--- a/2_Planning/CRONOGRAMA_GENERAL_ABB_Actualizado_2026-06-09.xlsx
+++ b/2_Planning/CRONOGRAMA_GENERAL_ABB_Actualizado_2026-06-09.xlsx
@@ -22,12 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MMM-YYYY"/>
-    <numFmt numFmtId="166" formatCode="$#,##0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="63">
+  <fonts count="67">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -389,8 +388,29 @@
       <color rgb="001F4E79"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00375623"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="43">
+  <fills count="44">
     <fill>
       <patternFill/>
     </fill>
@@ -602,8 +622,13 @@
         <fgColor rgb="00F0F8FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -723,11 +748,67 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="284">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1203,7 +1284,7 @@
     <xf numFmtId="0" fontId="3" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="33" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="27" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1215,7 +1296,7 @@
     <xf numFmtId="0" fontId="60" fillId="27" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="40" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1317,16 +1398,16 @@
     <xf numFmtId="0" fontId="7" fillId="41" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="41" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="41" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="26" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="26" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1341,28 +1422,28 @@
     <xf numFmtId="0" fontId="7" fillId="42" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="42" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="42" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="25" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="35" fillId="25" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="35" fillId="25" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1371,7 +1452,149 @@
     <xf numFmtId="0" fontId="61" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="35" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="34" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="27" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="23" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="43" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="34" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="27" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="39" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="41" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="21" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="26" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="42" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="19" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="35" fillId="25" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -18160,7 +18383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="B1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -18576,8 +18799,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="122" t="inlineStr">
         <is>
@@ -18733,321 +18954,1321 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="128" t="inlineStr">
-        <is>
-          <t>FREEZING POINTS — REGISTRO Y SEGUIMIENTO  |  27-MAY-2026 → ACTUALIZADO 09-JUN-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="129" t="inlineStr">
-        <is>
-          <t>Un cambio post-FP requiere Nota de Cambio + impacto costo/plazo. FP-P1 y FP-P2 actualizados per Cronograma ABB RevA (MS Project 27-MAY-2026 → ACTUALIZADO 09-JUN-2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="8" customHeight="1"/>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="130" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="234" t="inlineStr">
+        <is>
+          <t>FREEZING POINTS CORREGIDOS — PG-001 Rev A  |  Fuente: 5155-00-0009-VE-CO-PG-001_A.mpp  |  ABB 26-MAY-2026  |  Actualizado: 09-JUN-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="235" t="inlineStr">
+        <is>
+          <t>MPP contiene 20 FPs por equipo/nivel ingeniería. Correcciones críticas vs Excel previo: FP-S3-3 era 31-AGO → ahora 26-OCT (+56d) | FP-S3/S4 Sala ID era AGO → ahora 06-OCT (+39-53d) | ★ ÚLTIMO FP ABB REAL: Ductos barras 26-OCT-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SALA #3 BT — FREEZING POINTS POR EQUIPO (OC 4508944971)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="237" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C5" s="130" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="D5" s="130" t="inlineStr">
-        <is>
-          <t>Freezing Point</t>
-        </is>
-      </c>
-      <c r="E5" s="130" t="inlineStr">
-        <is>
-          <t>Fecha Plan</t>
-        </is>
-      </c>
-      <c r="F5" s="130" t="inlineStr">
+      <c r="B5" s="237" t="inlineStr">
+        <is>
+          <t>ID FP</t>
+        </is>
+      </c>
+      <c r="C5" s="237" t="inlineStr">
+        <is>
+          <t>Descripción FP</t>
+        </is>
+      </c>
+      <c r="D5" s="237" t="inlineStr">
+        <is>
+          <t>Fecha MPP</t>
+        </is>
+      </c>
+      <c r="E5" s="237" t="inlineStr">
+        <is>
+          <t>Δ vs Excel previo</t>
+        </is>
+      </c>
+      <c r="F5" s="237" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G5" s="130" t="inlineStr">
+      <c r="G5" s="237" t="inlineStr">
+        <is>
+          <t>OC / Sala</t>
+        </is>
+      </c>
+      <c r="H5" s="237" t="inlineStr">
         <is>
           <t>Impacto si demora</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="B6" s="131" t="n">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="238" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="132" t="inlineStr">
+      <c r="B6" s="239" t="inlineStr">
+        <is>
+          <t>FP-S3/Tab.Aux-IB</t>
+        </is>
+      </c>
+      <c r="C6" s="240" t="inlineStr">
+        <is>
+          <t>IB Tableros Auxiliares SE#3 (102-DP-001, LP-001/002, DP-001-TRA)</t>
+        </is>
+      </c>
+      <c r="D6" s="241" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="E6" s="242" t="inlineStr">
+        <is>
+          <t>-9d</t>
+        </is>
+      </c>
+      <c r="F6" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G6" s="243" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H6" s="244" t="inlineStr">
+        <is>
+          <t>Gatilla acopio materiales Tab.Aux → Fabricación Nov</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="238" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="239" t="inlineStr">
+        <is>
+          <t>FP-S3/Dr.BT-IB</t>
+        </is>
+      </c>
+      <c r="C7" s="240" t="inlineStr">
+        <is>
+          <t>IB Drives BT — 102-DP-VFD-24210A/B/C</t>
+        </is>
+      </c>
+      <c r="D7" s="241" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="245" t="inlineStr">
+        <is>
+          <t>-4d</t>
+        </is>
+      </c>
+      <c r="F7" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G7" s="243" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H7" s="244" t="inlineStr">
+        <is>
+          <t>OC VFDs Finlandia (lead ~4m) → Entrega Enero 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="246" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/CCM-IB</t>
+        </is>
+      </c>
+      <c r="C8" s="189" t="inlineStr">
+        <is>
+          <t>IB CCM-005 / CCM-006 / CCM-007 (todos el mismo día)</t>
+        </is>
+      </c>
+      <c r="D8" s="246" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="E8" s="245" t="inlineStr">
+        <is>
+          <t>+3d</t>
+        </is>
+      </c>
+      <c r="F8" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G8" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H8" s="248" t="inlineStr">
+        <is>
+          <t>OC ductos barras Turquía (lead 6m). CADENA CRÍTICA — 1d demora = impacto en despacho</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="238" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="239" t="inlineStr">
+        <is>
+          <t>FP-S3/UPS-IB</t>
+        </is>
+      </c>
+      <c r="C9" s="240" t="inlineStr">
+        <is>
+          <t>IB Rectificadores/UPS/Baterías — 102-UPS-001A/B, VCC-001A/B</t>
+        </is>
+      </c>
+      <c r="D9" s="241" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="245" t="inlineStr">
+        <is>
+          <t>+4d</t>
+        </is>
+      </c>
+      <c r="F9" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G9" s="243" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H9" s="244" t="inlineStr">
+        <is>
+          <t>Gatilla compra y acopio materiales → Fabricación Nov</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="238" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="239" t="inlineStr">
+        <is>
+          <t>FP-S3/Tab.Aux-ID</t>
+        </is>
+      </c>
+      <c r="C10" s="240" t="inlineStr">
+        <is>
+          <t>ID Tableros Auxiliares SE#3</t>
+        </is>
+      </c>
+      <c r="D10" s="241" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="242" t="inlineStr">
+        <is>
+          <t>-25d</t>
+        </is>
+      </c>
+      <c r="F10" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G10" s="243" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H10" s="244" t="inlineStr">
+        <is>
+          <t>Inicio fabricación tableros auxiliares. Entrega shelterista: Ene 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="238" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="239" t="inlineStr">
+        <is>
+          <t>FP-S3/Sala3-IB</t>
+        </is>
+      </c>
+      <c r="C11" s="240" t="inlineStr">
+        <is>
+          <t>IB Sala Eléctrica #3 — BUILDING (Layout + dimensiones + accesos)</t>
+        </is>
+      </c>
+      <c r="D11" s="241" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="242" t="inlineStr">
+        <is>
+          <t>+18d</t>
+        </is>
+      </c>
+      <c r="F11" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G11" s="243" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H11" s="244" t="inlineStr">
+        <is>
+          <t>Congela: dimensiones sala, acometidas trafo, disposición equipos S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="246" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/CCM005-ID</t>
+        </is>
+      </c>
+      <c r="C12" s="189" t="inlineStr">
+        <is>
+          <t>ID CCM-005 — Ingeniería de Detalle completa y aprobada</t>
+        </is>
+      </c>
+      <c r="D12" s="246" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E12" s="245" t="inlineStr">
+        <is>
+          <t>-2d</t>
+        </is>
+      </c>
+      <c r="F12" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G12" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H12" s="248" t="inlineStr">
+        <is>
+          <t>Inicio compra materiales secundarios CCM-005 → Fabricación Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="246" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/CCM006-ID</t>
+        </is>
+      </c>
+      <c r="C13" s="189" t="inlineStr">
+        <is>
+          <t>ID CCM-006 — Ingeniería de Detalle completa y aprobada</t>
+        </is>
+      </c>
+      <c r="D13" s="246" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="245" t="inlineStr">
+        <is>
+          <t>+3d</t>
+        </is>
+      </c>
+      <c r="F13" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G13" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H13" s="248" t="inlineStr">
+        <is>
+          <t>Inicio compra materiales secundarios CCM-006 → Fabricación Nov</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="246" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/CCM007-ID</t>
+        </is>
+      </c>
+      <c r="C14" s="189" t="inlineStr">
+        <is>
+          <t>ID CCM-007 — Ingeniería de Detalle completa y aprobada</t>
+        </is>
+      </c>
+      <c r="D14" s="246" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="245" t="inlineStr">
+        <is>
+          <t>+5d</t>
+        </is>
+      </c>
+      <c r="F14" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G14" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H14" s="248" t="inlineStr">
+        <is>
+          <t>Último FP CCM → Fabricación CCM-007 comienza Nov 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="246" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/Sala3-ID</t>
+        </is>
+      </c>
+      <c r="C15" s="189" t="inlineStr">
+        <is>
+          <t>★ ID Sala Eléctrica #3 — BUILDING (Planos constructivos + instalación)</t>
+        </is>
+      </c>
+      <c r="D15" s="246" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="249" t="inlineStr">
+        <is>
+          <t>+36d</t>
+        </is>
+      </c>
+      <c r="F15" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G15" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H15" s="248" t="inlineStr">
+        <is>
+          <t>Inicio fabricación sala → Construcción base Oct-Dic 2026. +36d vs Excel previo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="246" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="246" t="inlineStr">
+        <is>
+          <t>FP-S3/DB-FP</t>
+        </is>
+      </c>
+      <c r="C16" s="189" t="inlineStr">
+        <is>
+          <t>★★★ Ductos de Barras SE#3 — ÚLTIMO FP ABSOLUTO DEL PROYECTO ABB</t>
+        </is>
+      </c>
+      <c r="D16" s="246" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="249" t="inlineStr">
+        <is>
+          <t>+56d</t>
+        </is>
+      </c>
+      <c r="F16" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G16" s="247" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H16" s="248" t="inlineStr">
+        <is>
+          <t>ÚLTIMO FP REAL: Congela diseño ductos → Fabricación Tur/Oct-Ene → Despacho Ene 2027. +56d vs Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SALA #4 MT — FREEZING POINTS POR EQUIPO (OC 4508944973)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="237" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="237" t="inlineStr">
+        <is>
+          <t>ID FP</t>
+        </is>
+      </c>
+      <c r="C19" s="237" t="inlineStr">
+        <is>
+          <t>Descripción FP</t>
+        </is>
+      </c>
+      <c r="D19" s="237" t="inlineStr">
+        <is>
+          <t>Fecha MPP</t>
+        </is>
+      </c>
+      <c r="E19" s="237" t="inlineStr">
+        <is>
+          <t>Δ vs Excel previo</t>
+        </is>
+      </c>
+      <c r="F19" s="237" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="G19" s="237" t="inlineStr">
+        <is>
+          <t>OC / Sala</t>
+        </is>
+      </c>
+      <c r="H19" s="237" t="inlineStr">
+        <is>
+          <t>Impacto si demora</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="251" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Celdas-IB</t>
+        </is>
+      </c>
+      <c r="C20" s="193" t="inlineStr">
+        <is>
+          <t>IB Celdas MT Unigear 13.2/6.6kV (TGMT-001/002)</t>
+        </is>
+      </c>
+      <c r="D20" s="253" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
+      <c r="E20" s="245" t="inlineStr">
+        <is>
+          <t>-3d</t>
+        </is>
+      </c>
+      <c r="F20" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G20" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H20" s="255" t="inlineStr">
+        <is>
+          <t>OC Celdas MT Turquía (lead 6m) → Entrega Dic 2026. -3d vs Excel ≈ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="251" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Tab.Aux-IB</t>
+        </is>
+      </c>
+      <c r="C21" s="193" t="inlineStr">
+        <is>
+          <t>IB Tableros Auxiliares SE#4 (102-DP-101, DP-101UPS, DP-101VCC)</t>
+        </is>
+      </c>
+      <c r="D21" s="253" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="E21" s="245" t="inlineStr">
+        <is>
+          <t>-2d</t>
+        </is>
+      </c>
+      <c r="F21" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G21" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H21" s="255" t="inlineStr">
+        <is>
+          <t>Gatilla acopio materiales Tab.Aux → Fabricación Nov</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="251" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Dr.MT-IB</t>
+        </is>
+      </c>
+      <c r="C22" s="193" t="inlineStr">
+        <is>
+          <t>IB Drives MT — 102-DP-VFD-23310A/B/C</t>
+        </is>
+      </c>
+      <c r="D22" s="253" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="E22" s="245" t="inlineStr">
+        <is>
+          <t>+3d</t>
+        </is>
+      </c>
+      <c r="F22" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G22" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H22" s="255" t="inlineStr">
+        <is>
+          <t>OC VFDs MT China (lead 4-5m) → Entrega Feb 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="251" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Tab.Aux-ID</t>
+        </is>
+      </c>
+      <c r="C23" s="193" t="inlineStr">
+        <is>
+          <t>ID Tableros Auxiliares SE#4</t>
+        </is>
+      </c>
+      <c r="D23" s="253" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="242" t="inlineStr">
+        <is>
+          <t>-25d</t>
+        </is>
+      </c>
+      <c r="F23" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G23" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H23" s="255" t="inlineStr">
+        <is>
+          <t>Inicio fabricación tableros auxiliares → Entrega shelterista Ene 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="251" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Sala4-IB</t>
+        </is>
+      </c>
+      <c r="C24" s="193" t="inlineStr">
+        <is>
+          <t>IB Sala Eléctrica #4 — BUILDING (Layout + dimensiones + accesos)</t>
+        </is>
+      </c>
+      <c r="D24" s="253" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="E24" s="242" t="inlineStr">
+        <is>
+          <t>+25d</t>
+        </is>
+      </c>
+      <c r="F24" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G24" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H24" s="255" t="inlineStr">
+        <is>
+          <t>Congela: dimensiones sala MT, acometidas celdas, disposición equipos. +25d vs Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="251" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Celdas-ID</t>
+        </is>
+      </c>
+      <c r="C25" s="193" t="inlineStr">
+        <is>
+          <t>ID Celdas MT Unigear — Ingeniería de Detalle aprobada</t>
+        </is>
+      </c>
+      <c r="D25" s="253" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="E25" s="242" t="inlineStr">
+        <is>
+          <t>-11d</t>
+        </is>
+      </c>
+      <c r="F25" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G25" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H25" s="255" t="inlineStr">
+        <is>
+          <t>Inicio compra materiales secundarios → Fabricación Sep-Nov. -11d vs Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="251" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="252" t="inlineStr">
+        <is>
+          <t>FP-S4/Sala4-ID</t>
+        </is>
+      </c>
+      <c r="C26" s="193" t="inlineStr">
+        <is>
+          <t>★ ID Sala Eléctrica #4 — BUILDING (Planos constructivos + instalación)</t>
+        </is>
+      </c>
+      <c r="D26" s="253" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E26" s="249" t="inlineStr">
+        <is>
+          <t>+39d</t>
+        </is>
+      </c>
+      <c r="F26" s="242" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G26" s="254" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H26" s="255" t="inlineStr">
+        <is>
+          <t>Inicio fabricación sala → Construcción base Oct-Dic 2026. +39d vs Excel previo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RESUMEN COMPARATIVO: FECHAS EXCEL PREVIO vs MPP PG-001 Rev A (SIMPLIFICADO 8 FPs principales)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="257" t="inlineStr">
+        <is>
+          <t>ID (Excel)</t>
+        </is>
+      </c>
+      <c r="B29" s="257" t="inlineStr">
+        <is>
+          <t>FP Simplificado</t>
+        </is>
+      </c>
+      <c r="C29" s="257" t="inlineStr">
+        <is>
+          <t>Fecha Excel previo</t>
+        </is>
+      </c>
+      <c r="D29" s="257" t="inlineStr">
+        <is>
+          <t>Fecha MPP real</t>
+        </is>
+      </c>
+      <c r="E29" s="257" t="inlineStr">
+        <is>
+          <t>Diferencia</t>
+        </is>
+      </c>
+      <c r="F29" s="257" t="inlineStr">
+        <is>
+          <t>Veredicto</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="258" t="inlineStr">
         <is>
           <t>FP-P1</t>
         </is>
       </c>
-      <c r="D6" s="133" t="inlineStr">
-        <is>
-          <t>◆ Ing. Básica PMS</t>
-        </is>
-      </c>
-      <c r="E6" s="132" t="inlineStr">
+      <c r="B30" s="259" t="inlineStr">
+        <is>
+          <t>Ing. Básica PMS</t>
+        </is>
+      </c>
+      <c r="C30" s="260" t="inlineStr">
         <is>
           <t>21/08/2026</t>
         </is>
       </c>
-      <c r="F6" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G6" s="135" t="inlineStr">
-        <is>
-          <t>Demora FP-P1 → retrasa fabricación tableros + FAT Maqueta y FAT Tableros. Tiene holgura amplia pero buffer FAT Shelter se comprime</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="B7" s="131" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" s="132" t="inlineStr">
+      <c r="D30" s="261" t="inlineStr">
+        <is>
+          <t>sin cambio</t>
+        </is>
+      </c>
+      <c r="E30" s="262" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="263" t="inlineStr">
+        <is>
+          <t>PMS (otro MPP) — sin cambio</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="258" t="inlineStr">
         <is>
           <t>FP-P2</t>
         </is>
       </c>
-      <c r="D7" s="133" t="inlineStr">
-        <is>
-          <t>◆ Ing. Detalle + Procedimientos PMS</t>
-        </is>
-      </c>
-      <c r="E7" s="132" t="inlineStr">
+      <c r="B31" s="259" t="inlineStr">
+        <is>
+          <t>Ing. Detalle PMS</t>
+        </is>
+      </c>
+      <c r="C31" s="260" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="F7" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G7" s="135" t="inlineStr">
-        <is>
-          <t>Demora FP-P2 → FAT Tableros (29-ENE) se corre → Despacho (17-FEB) tarde → Montaje en Shelter tarde → FAT Integral Shelter tarde → impacto sobre FAT S#3</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="B8" s="131" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" s="132" t="inlineStr">
+      <c r="D31" s="261" t="inlineStr">
+        <is>
+          <t>sin cambio</t>
+        </is>
+      </c>
+      <c r="E31" s="262" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="263" t="inlineStr">
+        <is>
+          <t>PMS (otro MPP) — sin cambio</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="258" t="inlineStr">
         <is>
           <t>FP-S4-1</t>
         </is>
       </c>
-      <c r="D8" s="133" t="inlineStr">
-        <is>
-          <t>◆ Ing. Básica Sala #4</t>
-        </is>
-      </c>
-      <c r="E8" s="132" t="inlineStr">
+      <c r="B32" s="259" t="inlineStr">
+        <is>
+          <t>IB Sala #4 (equipos)</t>
+        </is>
+      </c>
+      <c r="C32" s="260" t="inlineStr">
         <is>
           <t>26/06/2026</t>
         </is>
       </c>
-      <c r="F8" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G8" s="135" t="inlineStr">
-        <is>
-          <t>Demora OC Turquía → celdas llegan tarde → FAT S4 tarde → Despacho S4 tarde (holgura 81d actual)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="B9" s="131" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" s="132" t="inlineStr">
+      <c r="D32" s="264" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
+      <c r="E32" s="245" t="inlineStr">
+        <is>
+          <t>-3d</t>
+        </is>
+      </c>
+      <c r="F32" s="263" t="inlineStr">
+        <is>
+          <t>≈OK — Celdas MT IB 23-JUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="258" t="inlineStr">
+        <is>
+          <t>FP-S4-1</t>
+        </is>
+      </c>
+      <c r="B33" s="259" t="inlineStr">
+        <is>
+          <t>IB Sala #4 (building)</t>
+        </is>
+      </c>
+      <c r="C33" s="260" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
+      <c r="D33" s="264" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="E33" s="242" t="inlineStr">
+        <is>
+          <t>+25d</t>
+        </is>
+      </c>
+      <c r="F33" s="265" t="inlineStr">
+        <is>
+          <t>⚠ REVISAR — Sala IB FP 21-JUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="258" t="inlineStr">
         <is>
           <t>FP-S4-2</t>
         </is>
       </c>
-      <c r="D9" s="133" t="inlineStr">
-        <is>
-          <t>◆ Ing. Detalle Sala #4</t>
-        </is>
-      </c>
-      <c r="E9" s="132" t="inlineStr">
+      <c r="B34" s="259" t="inlineStr">
+        <is>
+          <t>ID Sala #4 (Celdas MT)</t>
+        </is>
+      </c>
+      <c r="C34" s="260" t="inlineStr">
         <is>
           <t>14/08/2026</t>
         </is>
       </c>
-      <c r="F9" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G9" s="135" t="inlineStr">
-        <is>
-          <t>Demora → montaje Shelter S4 tarde → FAT S4 tarde</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="B10" s="131" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="132" t="inlineStr">
+      <c r="D34" s="264" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="E34" s="242" t="inlineStr">
+        <is>
+          <t>-11d</t>
+        </is>
+      </c>
+      <c r="F34" s="265" t="inlineStr">
+        <is>
+          <t>⚠ Celdas ID es 03-AGO (-11d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="258" t="inlineStr">
+        <is>
+          <t>FP-S4-2</t>
+        </is>
+      </c>
+      <c r="B35" s="259" t="inlineStr">
+        <is>
+          <t>ID Sala #4 (building)</t>
+        </is>
+      </c>
+      <c r="C35" s="260" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="D35" s="266" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E35" s="249" t="inlineStr">
+        <is>
+          <t>+53d</t>
+        </is>
+      </c>
+      <c r="F35" s="267" t="inlineStr">
+        <is>
+          <t>🔴 CRÍTICO: Sala ID es 06-OCT (+53d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="258" t="inlineStr">
         <is>
           <t>FP-S4-3</t>
         </is>
       </c>
-      <c r="D10" s="133" t="inlineStr">
-        <is>
-          <t>◆ Ing. Constructiva Sala #4  ← CIERRA ING. S4</t>
-        </is>
-      </c>
-      <c r="E10" s="132" t="inlineStr">
+      <c r="B36" s="259" t="inlineStr">
+        <is>
+          <t>IC Sala #4 (→ ID building)</t>
+        </is>
+      </c>
+      <c r="C36" s="260" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="F10" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G10" s="135" t="inlineStr">
-        <is>
-          <t>Demora directa sobre montaje Shelter S4 → FAT S4 tarde. Margen S4: 81d sobre P6</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="B11" s="136" t="n">
-        <v>6</v>
-      </c>
-      <c r="C11" s="137" t="inlineStr">
+      <c r="D36" s="266" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="249" t="inlineStr">
+        <is>
+          <t>+39d</t>
+        </is>
+      </c>
+      <c r="F36" s="267" t="inlineStr">
+        <is>
+          <t>🔴 CRÍTICO: +39 días — usar 06-OCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="258" t="inlineStr">
         <is>
           <t>FP-S3-1</t>
         </is>
       </c>
-      <c r="D11" s="138" t="inlineStr">
-        <is>
-          <t>◆ Ing. Básica Sala #3</t>
-        </is>
-      </c>
-      <c r="E11" s="137" t="inlineStr">
+      <c r="B37" s="259" t="inlineStr">
+        <is>
+          <t>IB Sala #3 (CCMs)</t>
+        </is>
+      </c>
+      <c r="C37" s="260" t="inlineStr">
         <is>
           <t>03/07/2026</t>
         </is>
       </c>
-      <c r="F11" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G11" s="139" t="inlineStr">
-        <is>
-          <t>1 día de demora → OC Turquía tarde → ductos llegan tarde → FAT S3 tarde → PENALIDAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="B12" s="136" t="n">
-        <v>7</v>
-      </c>
-      <c r="C12" s="137" t="inlineStr">
+      <c r="D37" s="264" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="E37" s="245" t="inlineStr">
+        <is>
+          <t>+3d</t>
+        </is>
+      </c>
+      <c r="F37" s="263" t="inlineStr">
+        <is>
+          <t>≈OK — CCMs IB FP 06-JUL (+3d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="258" t="inlineStr">
+        <is>
+          <t>FP-S3-1</t>
+        </is>
+      </c>
+      <c r="B38" s="259" t="inlineStr">
+        <is>
+          <t>IB Sala #3 (building)</t>
+        </is>
+      </c>
+      <c r="C38" s="260" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="D38" s="264" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="E38" s="242" t="inlineStr">
+        <is>
+          <t>+18d</t>
+        </is>
+      </c>
+      <c r="F38" s="265" t="inlineStr">
+        <is>
+          <t>⚠ REVISAR — Sala IB FP 21-JUL (+18d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="258" t="inlineStr">
         <is>
           <t>FP-S3-2</t>
         </is>
       </c>
-      <c r="D12" s="138" t="inlineStr">
-        <is>
-          <t>◆ Ing. Detalle Sala #3</t>
-        </is>
-      </c>
-      <c r="E12" s="137" t="inlineStr">
+      <c r="B39" s="259" t="inlineStr">
+        <is>
+          <t>ID Sala #3 (CCMs)</t>
+        </is>
+      </c>
+      <c r="C39" s="260" t="inlineStr">
         <is>
           <t>14/08/2026</t>
         </is>
       </c>
-      <c r="F12" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G12" s="139" t="inlineStr">
-        <is>
-          <t>Demora → fabricación CCMs tarde → ensayos tarde → FAT S#3 tarde → Despacho tarde → PENALIDAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="B13" s="136" t="n">
-        <v>8</v>
-      </c>
-      <c r="C13" s="137" t="inlineStr">
+      <c r="D39" s="264" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="E39" s="245" t="inlineStr">
+        <is>
+          <t>-2d</t>
+        </is>
+      </c>
+      <c r="F39" s="263" t="inlineStr">
+        <is>
+          <t>≈OK — CCM-005 ID 12-AGO (-2d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="258" t="inlineStr">
+        <is>
+          <t>FP-S3-2</t>
+        </is>
+      </c>
+      <c r="B40" s="259" t="inlineStr">
+        <is>
+          <t>ID Sala #3 (building)</t>
+        </is>
+      </c>
+      <c r="C40" s="260" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="D40" s="266" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E40" s="249" t="inlineStr">
+        <is>
+          <t>+53d</t>
+        </is>
+      </c>
+      <c r="F40" s="267" t="inlineStr">
+        <is>
+          <t>🔴 CRÍTICO: Sala ID es 06-OCT (+53d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="258" t="inlineStr">
         <is>
           <t>FP-S3-3</t>
         </is>
       </c>
-      <c r="D13" s="138" t="inlineStr">
-        <is>
-          <t>◆ Ing. Constructiva S#3  ★ ÚLTIMO FP ABB</t>
-        </is>
-      </c>
-      <c r="E13" s="137" t="inlineStr">
+      <c r="B41" s="259" t="inlineStr">
+        <is>
+          <t>IC/Último FP S3 (Sala)</t>
+        </is>
+      </c>
+      <c r="C41" s="260" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="F13" s="134" t="inlineStr">
-        <is>
-          <t>Pendiente ⚠</t>
-        </is>
-      </c>
-      <c r="G13" s="139" t="inlineStr">
-        <is>
-          <t>1 semana late → montaje Shelter S3 late → FAT 1 semana late → Despacho 1 semana late → PENALIDAD 1%/semana</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="140" t="inlineStr">
-        <is>
-          <t>⚠ FP-P1 y FP-P2 actualizados: FP-P1 era 19-JUN → ahora 21-AGO  |  FP-P2 era 31-JUL → ahora 23-OCT  |  Per Cronograma MS Project ABB RevA (E-2611027, 27-MAY-2026 → ACTUALIZADO 09-JUN-2026)</t>
+      <c r="D41" s="266" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="E41" s="249" t="inlineStr">
+        <is>
+          <t>+36d</t>
+        </is>
+      </c>
+      <c r="F41" s="267" t="inlineStr">
+        <is>
+          <t>🔴 CRÍTICO: Sala ID es 06-OCT (+36d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="258" t="inlineStr">
+        <is>
+          <t>FP-S3-3</t>
+        </is>
+      </c>
+      <c r="B42" s="259" t="inlineStr">
+        <is>
+          <t>★ ÚLTIMO FP REAL (Ductos)</t>
+        </is>
+      </c>
+      <c r="C42" s="260" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="D42" s="266" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="249" t="inlineStr">
+        <is>
+          <t>+56d</t>
+        </is>
+      </c>
+      <c r="F42" s="267" t="inlineStr">
+        <is>
+          <t>🔴 CRÍTICO: Ductos 26-OCT (+56 DÍAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="44" customHeight="1">
+      <c r="A44" s="268" t="inlineStr">
+        <is>
+          <t>⚠ ACCIÓN INMEDIATA: El ÚLTIMO FP real del proyecto es Ductos de barras el 26-OCT-2026 (no el 31-AGO-2026 que figuraba antes). El plazo hasta el último FP se extendió +56 días, lo que puede afectar las fechas de despacho si no se gestionan los proveedores de Turquía. | Sala eléctrica ID FPs (S3 y S4) = 06-OCT-2026. | Revisar lead times de fabricación con el nuevo cronograma.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B1:G1"/>
+  <mergeCells count="6">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19059,7 +20280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="B1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -19651,6 +20872,11 @@
           <t>ESTADO DEL PROYECTO — INFORME DE AVANCE N°1  |  ABB  |  Período: Mayo 2026  |  Actualizado: 09-JUN-2026</t>
         </is>
       </c>
+      <c r="B1" s="269" t="n"/>
+      <c r="C1" s="269" t="n"/>
+      <c r="D1" s="269" t="n"/>
+      <c r="E1" s="269" t="n"/>
+      <c r="F1" s="270" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="160" t="inlineStr">
@@ -19658,6 +20884,11 @@
           <t>Fuente: R-2631036 Informe de Avance N°1 (04-JUN-2026)  |  Cronograma Oficial: 5155-00-0009-VE-CO-PG-001 Rev A  |  R-2631036 Cronograma de Certificaciones Rev A  |  PM ABB: Rodrigo Mack</t>
         </is>
       </c>
+      <c r="B2" s="271" t="n"/>
+      <c r="C2" s="271" t="n"/>
+      <c r="D2" s="271" t="n"/>
+      <c r="E2" s="271" t="n"/>
+      <c r="F2" s="272" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="161" t="inlineStr">
@@ -19665,6 +20896,11 @@
           <t>A. RESUMEN DE ESTADO — AVANCE MAYO 2026</t>
         </is>
       </c>
+      <c r="B4" s="271" t="n"/>
+      <c r="C4" s="271" t="n"/>
+      <c r="D4" s="271" t="n"/>
+      <c r="E4" s="271" t="n"/>
+      <c r="F4" s="272" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="162" t="inlineStr">
@@ -19716,6 +20952,7 @@
           <t>Ingeniería Básica iniciada en todos los equipos. RevA en elaboración</t>
         </is>
       </c>
+      <c r="F6" s="272" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="163" t="inlineStr">
@@ -19743,6 +20980,7 @@
           <t>Arquitectura+I/O+Planos Constructivos RevA iniciados</t>
         </is>
       </c>
+      <c r="F7" s="272" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="163" t="inlineStr">
@@ -19770,6 +21008,7 @@
           <t>Aguardan aprobación IB. OC Turquía/China/Finlandia no emitidas aún</t>
         </is>
       </c>
+      <c r="F8" s="272" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="163" t="inlineStr">
@@ -19797,6 +21036,7 @@
           <t>Sin actividades de fabricación en el período Mayo 2026</t>
         </is>
       </c>
+      <c r="F9" s="272" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="163" t="inlineStr">
@@ -19824,6 +21064,7 @@
           <t>En preparación para CCMs, tableros MT/BT, VFDs</t>
         </is>
       </c>
+      <c r="F10" s="272" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="163" t="inlineStr">
@@ -19851,6 +21092,7 @@
           <t>Primer pago S3+S4: Jun 2026. Ver hoja 6_Cert_Mensual</t>
         </is>
       </c>
+      <c r="F11" s="272" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="163" t="inlineStr">
@@ -19878,6 +21120,7 @@
           <t>5155-00-0009-VE-CO-PG-001_A.mpp emitido 26-MAY-2026 por PM Rodrigo Mack</t>
         </is>
       </c>
+      <c r="F12" s="272" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="163" t="inlineStr">
@@ -19905,6 +21148,7 @@
           <t>R-2631036 Informe Avance N°1 emitido 04-JUN-2026</t>
         </is>
       </c>
+      <c r="F13" s="272" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="175" t="inlineStr">
@@ -19912,6 +21156,11 @@
           <t>B. PENDIENTES CRÍTICOS — INFORMACIÓN REQUERIDA A AESA</t>
         </is>
       </c>
+      <c r="B15" s="271" t="n"/>
+      <c r="C15" s="271" t="n"/>
+      <c r="D15" s="271" t="n"/>
+      <c r="E15" s="271" t="n"/>
+      <c r="F15" s="272" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="176" t="inlineStr">
@@ -19946,7 +21195,7 @@
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="177" t="n">
+      <c r="A17" s="273" t="n">
         <v>46178</v>
       </c>
       <c r="B17" s="178" t="inlineStr">
@@ -19976,7 +21225,7 @@
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="181" t="n">
+      <c r="A18" s="274" t="n">
         <v>46191</v>
       </c>
       <c r="B18" s="182" t="inlineStr">
@@ -20006,7 +21255,7 @@
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="181" t="n">
+      <c r="A19" s="274" t="n">
         <v>46203</v>
       </c>
       <c r="B19" s="182" t="inlineStr">
@@ -20036,7 +21285,7 @@
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="181" t="n">
+      <c r="A20" s="274" t="n">
         <v>46223</v>
       </c>
       <c r="B20" s="185" t="inlineStr">
@@ -20071,6 +21320,11 @@
           <t>C. ALCANCE CONFIRMADO — SALAS ELÉCTRICAS (según Informe N°1)</t>
         </is>
       </c>
+      <c r="B22" s="271" t="n"/>
+      <c r="C22" s="271" t="n"/>
+      <c r="D22" s="271" t="n"/>
+      <c r="E22" s="271" t="n"/>
+      <c r="F22" s="272" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="162" t="inlineStr">
@@ -20189,8 +21443,8 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E10:F10"/>
     <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E10:F10"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="A15:F15"/>
@@ -20241,6 +21495,25 @@
           <t>CRONOGRAMA DE CERTIFICACIONES MENSUAL — OC S3 + OC S4  |  Actualizado: 09-JUN-2026  |  Fuente: R-2631036 Cron. Certificaciones Rev A</t>
         </is>
       </c>
+      <c r="B1" s="269" t="n"/>
+      <c r="C1" s="269" t="n"/>
+      <c r="D1" s="269" t="n"/>
+      <c r="E1" s="269" t="n"/>
+      <c r="F1" s="269" t="n"/>
+      <c r="G1" s="269" t="n"/>
+      <c r="H1" s="269" t="n"/>
+      <c r="I1" s="269" t="n"/>
+      <c r="J1" s="269" t="n"/>
+      <c r="K1" s="269" t="n"/>
+      <c r="L1" s="269" t="n"/>
+      <c r="M1" s="269" t="n"/>
+      <c r="N1" s="269" t="n"/>
+      <c r="O1" s="269" t="n"/>
+      <c r="P1" s="269" t="n"/>
+      <c r="Q1" s="269" t="n"/>
+      <c r="R1" s="269" t="n"/>
+      <c r="S1" s="269" t="n"/>
+      <c r="T1" s="270" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="201" t="inlineStr">
@@ -20248,6 +21521,25 @@
           <t>Hito 1:10% envío IB  |  Hito 2:10% aprob. IB  |  Hito 3:20% FAT  |  Hito 4:25% Acopio  |  Hito 5:30% Entrega  |  Hito 6:5% DataBook  |  Hito 7:100% Repuestos (separado)  |  Totales excluyen repuestos (ítems 10-60)</t>
         </is>
       </c>
+      <c r="B2" s="271" t="n"/>
+      <c r="C2" s="271" t="n"/>
+      <c r="D2" s="271" t="n"/>
+      <c r="E2" s="271" t="n"/>
+      <c r="F2" s="271" t="n"/>
+      <c r="G2" s="271" t="n"/>
+      <c r="H2" s="271" t="n"/>
+      <c r="I2" s="271" t="n"/>
+      <c r="J2" s="271" t="n"/>
+      <c r="K2" s="271" t="n"/>
+      <c r="L2" s="271" t="n"/>
+      <c r="M2" s="271" t="n"/>
+      <c r="N2" s="271" t="n"/>
+      <c r="O2" s="271" t="n"/>
+      <c r="P2" s="271" t="n"/>
+      <c r="Q2" s="271" t="n"/>
+      <c r="R2" s="271" t="n"/>
+      <c r="S2" s="271" t="n"/>
+      <c r="T2" s="272" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="202" t="inlineStr">
@@ -20359,6 +21651,25 @@
           <t>OC S3 — 4508944971  |  Sala 3 BT  |  Total: USD 8,027,904</t>
         </is>
       </c>
+      <c r="B4" s="271" t="n"/>
+      <c r="C4" s="271" t="n"/>
+      <c r="D4" s="271" t="n"/>
+      <c r="E4" s="271" t="n"/>
+      <c r="F4" s="271" t="n"/>
+      <c r="G4" s="271" t="n"/>
+      <c r="H4" s="271" t="n"/>
+      <c r="I4" s="271" t="n"/>
+      <c r="J4" s="271" t="n"/>
+      <c r="K4" s="271" t="n"/>
+      <c r="L4" s="271" t="n"/>
+      <c r="M4" s="271" t="n"/>
+      <c r="N4" s="271" t="n"/>
+      <c r="O4" s="271" t="n"/>
+      <c r="P4" s="271" t="n"/>
+      <c r="Q4" s="271" t="n"/>
+      <c r="R4" s="271" t="n"/>
+      <c r="S4" s="271" t="n"/>
+      <c r="T4" s="272" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="212" t="inlineStr">
@@ -20377,33 +21688,33 @@
           <t>VFD BT Bombas</t>
         </is>
       </c>
-      <c r="D5" s="215" t="n">
+      <c r="D5" s="275" t="n">
         <v>242508.12</v>
       </c>
       <c r="E5" s="216" t="n"/>
       <c r="F5" s="216" t="n"/>
-      <c r="G5" s="217" t="n">
+      <c r="G5" s="276" t="n">
         <v>24250.81</v>
       </c>
       <c r="H5" s="216" t="n"/>
       <c r="I5" s="216" t="n"/>
       <c r="J5" s="216" t="n"/>
       <c r="K5" s="216" t="n"/>
-      <c r="L5" s="217" t="n">
+      <c r="L5" s="276" t="n">
         <v>133379.47</v>
       </c>
       <c r="M5" s="216" t="n"/>
       <c r="N5" s="216" t="n"/>
       <c r="O5" s="216" t="n"/>
       <c r="P5" s="216" t="n"/>
-      <c r="Q5" s="217" t="n">
+      <c r="Q5" s="276" t="n">
         <v>72752.44</v>
       </c>
-      <c r="R5" s="217" t="n">
+      <c r="R5" s="276" t="n">
         <v>12125.41</v>
       </c>
       <c r="S5" s="216" t="n"/>
-      <c r="T5" s="218" t="n">
+      <c r="T5" s="277" t="n">
         <v>242508.13</v>
       </c>
     </row>
@@ -20424,37 +21735,37 @@
           <t>Tab. Distribución Tracing</t>
         </is>
       </c>
-      <c r="D6" s="215" t="n">
+      <c r="D6" s="275" t="n">
         <v>95632.73</v>
       </c>
       <c r="E6" s="216" t="n"/>
-      <c r="F6" s="217" t="n">
+      <c r="F6" s="276" t="n">
         <v>9563.27</v>
       </c>
-      <c r="G6" s="217" t="n">
+      <c r="G6" s="276" t="n">
         <v>9563.27</v>
       </c>
       <c r="H6" s="216" t="n"/>
       <c r="I6" s="216" t="n"/>
       <c r="J6" s="216" t="n"/>
-      <c r="K6" s="217" t="n">
+      <c r="K6" s="276" t="n">
         <v>23908.18</v>
       </c>
-      <c r="L6" s="217" t="n">
+      <c r="L6" s="276" t="n">
         <v>19126.55</v>
       </c>
       <c r="M6" s="216" t="n"/>
       <c r="N6" s="216" t="n"/>
       <c r="O6" s="216" t="n"/>
       <c r="P6" s="216" t="n"/>
-      <c r="Q6" s="217" t="n">
+      <c r="Q6" s="276" t="n">
         <v>28689.82</v>
       </c>
-      <c r="R6" s="217" t="n">
+      <c r="R6" s="276" t="n">
         <v>4781.64</v>
       </c>
       <c r="S6" s="216" t="n"/>
-      <c r="T6" s="218" t="n">
+      <c r="T6" s="277" t="n">
         <v>95632.73</v>
       </c>
     </row>
@@ -20475,37 +21786,37 @@
           <t>Tab. Serv. Aux. SE#3</t>
         </is>
       </c>
-      <c r="D7" s="215" t="n">
+      <c r="D7" s="275" t="n">
         <v>105885.06</v>
       </c>
       <c r="E7" s="216" t="n"/>
-      <c r="F7" s="217" t="n">
+      <c r="F7" s="276" t="n">
         <v>10588.51</v>
       </c>
-      <c r="G7" s="217" t="n">
+      <c r="G7" s="276" t="n">
         <v>10588.51</v>
       </c>
       <c r="H7" s="216" t="n"/>
       <c r="I7" s="216" t="n"/>
       <c r="J7" s="216" t="n"/>
-      <c r="K7" s="217" t="n">
+      <c r="K7" s="276" t="n">
         <v>26471.27</v>
       </c>
-      <c r="L7" s="217" t="n">
+      <c r="L7" s="276" t="n">
         <v>21177.01</v>
       </c>
       <c r="M7" s="216" t="n"/>
       <c r="N7" s="216" t="n"/>
       <c r="O7" s="216" t="n"/>
       <c r="P7" s="216" t="n"/>
-      <c r="Q7" s="217" t="n">
+      <c r="Q7" s="276" t="n">
         <v>31765.52</v>
       </c>
-      <c r="R7" s="217" t="n">
+      <c r="R7" s="276" t="n">
         <v>5294.25</v>
       </c>
       <c r="S7" s="216" t="n"/>
-      <c r="T7" s="218" t="n">
+      <c r="T7" s="277" t="n">
         <v>105885.07</v>
       </c>
     </row>
@@ -20526,37 +21837,37 @@
           <t>Tab. Distribución UPS</t>
         </is>
       </c>
-      <c r="D8" s="215" t="n">
+      <c r="D8" s="275" t="n">
         <v>63485.7</v>
       </c>
       <c r="E8" s="216" t="n"/>
-      <c r="F8" s="217" t="n">
+      <c r="F8" s="276" t="n">
         <v>6348.57</v>
       </c>
-      <c r="G8" s="217" t="n">
+      <c r="G8" s="276" t="n">
         <v>6348.57</v>
       </c>
       <c r="H8" s="216" t="n"/>
       <c r="I8" s="216" t="n"/>
       <c r="J8" s="216" t="n"/>
-      <c r="K8" s="217" t="n">
+      <c r="K8" s="276" t="n">
         <v>15871.43</v>
       </c>
-      <c r="L8" s="217" t="n">
+      <c r="L8" s="276" t="n">
         <v>12697.14</v>
       </c>
       <c r="M8" s="216" t="n"/>
       <c r="N8" s="216" t="n"/>
       <c r="O8" s="216" t="n"/>
       <c r="P8" s="216" t="n"/>
-      <c r="Q8" s="217" t="n">
+      <c r="Q8" s="276" t="n">
         <v>19045.71</v>
       </c>
-      <c r="R8" s="217" t="n">
+      <c r="R8" s="276" t="n">
         <v>3174.29</v>
       </c>
       <c r="S8" s="216" t="n"/>
-      <c r="T8" s="218" t="n">
+      <c r="T8" s="277" t="n">
         <v>63485.71</v>
       </c>
     </row>
@@ -20577,37 +21888,37 @@
           <t>Tab. Distribución Serv. Aux.</t>
         </is>
       </c>
-      <c r="D9" s="215" t="n">
+      <c r="D9" s="275" t="n">
         <v>96409.77</v>
       </c>
       <c r="E9" s="216" t="n"/>
-      <c r="F9" s="217" t="n">
+      <c r="F9" s="276" t="n">
         <v>9640.98</v>
       </c>
-      <c r="G9" s="217" t="n">
+      <c r="G9" s="276" t="n">
         <v>9640.98</v>
       </c>
       <c r="H9" s="216" t="n"/>
       <c r="I9" s="216" t="n"/>
       <c r="J9" s="216" t="n"/>
-      <c r="K9" s="217" t="n">
+      <c r="K9" s="276" t="n">
         <v>24102.44</v>
       </c>
-      <c r="L9" s="217" t="n">
+      <c r="L9" s="276" t="n">
         <v>19281.95</v>
       </c>
       <c r="M9" s="216" t="n"/>
       <c r="N9" s="216" t="n"/>
       <c r="O9" s="216" t="n"/>
       <c r="P9" s="216" t="n"/>
-      <c r="Q9" s="217" t="n">
+      <c r="Q9" s="276" t="n">
         <v>28922.93</v>
       </c>
-      <c r="R9" s="217" t="n">
+      <c r="R9" s="276" t="n">
         <v>4820.49</v>
       </c>
       <c r="S9" s="216" t="n"/>
-      <c r="T9" s="218" t="n">
+      <c r="T9" s="277" t="n">
         <v>96409.77</v>
       </c>
     </row>
@@ -20628,37 +21939,37 @@
           <t>Ducto Barras DB-007</t>
         </is>
       </c>
-      <c r="D10" s="215" t="n">
+      <c r="D10" s="275" t="n">
         <v>169501.43</v>
       </c>
       <c r="E10" s="216" t="n"/>
       <c r="F10" s="216" t="n"/>
-      <c r="G10" s="217" t="n">
+      <c r="G10" s="276" t="n">
         <v>16950.14</v>
       </c>
-      <c r="H10" s="217" t="n">
+      <c r="H10" s="276" t="n">
         <v>16950.14</v>
       </c>
       <c r="I10" s="216" t="n"/>
       <c r="J10" s="216" t="n"/>
       <c r="K10" s="216" t="n"/>
-      <c r="L10" s="217" t="n">
+      <c r="L10" s="276" t="n">
         <v>33900.29</v>
       </c>
       <c r="M10" s="216" t="n"/>
-      <c r="N10" s="217" t="n">
+      <c r="N10" s="276" t="n">
         <v>42375.36</v>
       </c>
       <c r="O10" s="216" t="n"/>
       <c r="P10" s="216" t="n"/>
-      <c r="Q10" s="217" t="n">
+      <c r="Q10" s="276" t="n">
         <v>50850.43</v>
       </c>
-      <c r="R10" s="217" t="n">
+      <c r="R10" s="276" t="n">
         <v>8475.07</v>
       </c>
       <c r="S10" s="216" t="n"/>
-      <c r="T10" s="218" t="n">
+      <c r="T10" s="277" t="n">
         <v>169501.43</v>
       </c>
     </row>
@@ -20679,37 +21990,37 @@
           <t>Ducto Barras DB-006</t>
         </is>
       </c>
-      <c r="D11" s="215" t="n">
+      <c r="D11" s="275" t="n">
         <v>182075.08</v>
       </c>
       <c r="E11" s="216" t="n"/>
       <c r="F11" s="216" t="n"/>
-      <c r="G11" s="217" t="n">
+      <c r="G11" s="276" t="n">
         <v>18207.51</v>
       </c>
-      <c r="H11" s="217" t="n">
+      <c r="H11" s="276" t="n">
         <v>18207.51</v>
       </c>
       <c r="I11" s="216" t="n"/>
       <c r="J11" s="216" t="n"/>
       <c r="K11" s="216" t="n"/>
-      <c r="L11" s="217" t="n">
+      <c r="L11" s="276" t="n">
         <v>36415.02</v>
       </c>
       <c r="M11" s="216" t="n"/>
-      <c r="N11" s="217" t="n">
+      <c r="N11" s="276" t="n">
         <v>45518.77</v>
       </c>
       <c r="O11" s="216" t="n"/>
       <c r="P11" s="216" t="n"/>
-      <c r="Q11" s="217" t="n">
+      <c r="Q11" s="276" t="n">
         <v>54622.52</v>
       </c>
-      <c r="R11" s="217" t="n">
+      <c r="R11" s="276" t="n">
         <v>9103.75</v>
       </c>
       <c r="S11" s="216" t="n"/>
-      <c r="T11" s="218" t="n">
+      <c r="T11" s="277" t="n">
         <v>182075.08</v>
       </c>
     </row>
@@ -20730,37 +22041,37 @@
           <t>Ducto Barras DB-005</t>
         </is>
       </c>
-      <c r="D12" s="215" t="n">
+      <c r="D12" s="275" t="n">
         <v>139094.32</v>
       </c>
       <c r="E12" s="216" t="n"/>
       <c r="F12" s="216" t="n"/>
-      <c r="G12" s="217" t="n">
+      <c r="G12" s="276" t="n">
         <v>13909.43</v>
       </c>
-      <c r="H12" s="217" t="n">
+      <c r="H12" s="276" t="n">
         <v>13909.43</v>
       </c>
       <c r="I12" s="216" t="n"/>
       <c r="J12" s="216" t="n"/>
       <c r="K12" s="216" t="n"/>
-      <c r="L12" s="217" t="n">
+      <c r="L12" s="276" t="n">
         <v>27818.86</v>
       </c>
       <c r="M12" s="216" t="n"/>
-      <c r="N12" s="217" t="n">
+      <c r="N12" s="276" t="n">
         <v>34773.58</v>
       </c>
       <c r="O12" s="216" t="n"/>
       <c r="P12" s="216" t="n"/>
-      <c r="Q12" s="217" t="n">
+      <c r="Q12" s="276" t="n">
         <v>41728.3</v>
       </c>
-      <c r="R12" s="217" t="n">
+      <c r="R12" s="276" t="n">
         <v>6954.72</v>
       </c>
       <c r="S12" s="216" t="n"/>
-      <c r="T12" s="218" t="n">
+      <c r="T12" s="277" t="n">
         <v>139094.32</v>
       </c>
     </row>
@@ -20781,7 +22092,7 @@
           <t>CCM 380/220V lote 1</t>
         </is>
       </c>
-      <c r="D13" s="215" t="n">
+      <c r="D13" s="275" t="n">
         <v>451298.47</v>
       </c>
       <c r="E13" s="216" t="n"/>
@@ -20791,21 +22102,21 @@
       <c r="I13" s="216" t="n"/>
       <c r="J13" s="216" t="n"/>
       <c r="K13" s="216" t="n"/>
-      <c r="L13" s="217" t="n">
+      <c r="L13" s="276" t="n">
         <v>293344.01</v>
       </c>
       <c r="M13" s="216" t="n"/>
       <c r="N13" s="216" t="n"/>
       <c r="O13" s="216" t="n"/>
       <c r="P13" s="216" t="n"/>
-      <c r="Q13" s="217" t="n">
+      <c r="Q13" s="276" t="n">
         <v>135389.54</v>
       </c>
-      <c r="R13" s="217" t="n">
+      <c r="R13" s="276" t="n">
         <v>22564.92</v>
       </c>
       <c r="S13" s="216" t="n"/>
-      <c r="T13" s="218" t="n">
+      <c r="T13" s="277" t="n">
         <v>451298.47</v>
       </c>
     </row>
@@ -20826,7 +22137,7 @@
           <t>CCM 380/220V lote 1</t>
         </is>
       </c>
-      <c r="D14" s="215" t="n">
+      <c r="D14" s="275" t="n">
         <v>492942.64</v>
       </c>
       <c r="E14" s="216" t="n"/>
@@ -20836,21 +22147,21 @@
       <c r="I14" s="216" t="n"/>
       <c r="J14" s="216" t="n"/>
       <c r="K14" s="216" t="n"/>
-      <c r="L14" s="217" t="n">
+      <c r="L14" s="276" t="n">
         <v>320412.72</v>
       </c>
       <c r="M14" s="216" t="n"/>
       <c r="N14" s="216" t="n"/>
       <c r="O14" s="216" t="n"/>
       <c r="P14" s="216" t="n"/>
-      <c r="Q14" s="217" t="n">
+      <c r="Q14" s="276" t="n">
         <v>147882.79</v>
       </c>
-      <c r="R14" s="217" t="n">
+      <c r="R14" s="276" t="n">
         <v>24647.13</v>
       </c>
       <c r="S14" s="216" t="n"/>
-      <c r="T14" s="218" t="n">
+      <c r="T14" s="277" t="n">
         <v>492942.64</v>
       </c>
     </row>
@@ -20871,7 +22182,7 @@
           <t>CCM 380/220V lote 1</t>
         </is>
       </c>
-      <c r="D15" s="215" t="n">
+      <c r="D15" s="275" t="n">
         <v>552737.98</v>
       </c>
       <c r="E15" s="216" t="n"/>
@@ -20881,21 +22192,21 @@
       <c r="I15" s="216" t="n"/>
       <c r="J15" s="216" t="n"/>
       <c r="K15" s="216" t="n"/>
-      <c r="L15" s="217" t="n">
+      <c r="L15" s="276" t="n">
         <v>359279.69</v>
       </c>
       <c r="M15" s="216" t="n"/>
       <c r="N15" s="216" t="n"/>
       <c r="O15" s="216" t="n"/>
       <c r="P15" s="216" t="n"/>
-      <c r="Q15" s="217" t="n">
+      <c r="Q15" s="276" t="n">
         <v>165821.39</v>
       </c>
-      <c r="R15" s="217" t="n">
+      <c r="R15" s="276" t="n">
         <v>27636.9</v>
       </c>
       <c r="S15" s="216" t="n"/>
-      <c r="T15" s="218" t="n">
+      <c r="T15" s="277" t="n">
         <v>552737.9800000001</v>
       </c>
     </row>
@@ -20916,37 +22227,37 @@
           <t>Sala Eléctrica N°3 BT</t>
         </is>
       </c>
-      <c r="D16" s="215" t="n">
+      <c r="D16" s="275" t="n">
         <v>622817.0699999999</v>
       </c>
       <c r="E16" s="216" t="n"/>
       <c r="F16" s="216" t="n"/>
-      <c r="G16" s="217" t="n">
+      <c r="G16" s="276" t="n">
         <v>62281.71</v>
       </c>
-      <c r="H16" s="217" t="n">
+      <c r="H16" s="276" t="n">
         <v>62281.71</v>
       </c>
       <c r="I16" s="216" t="n"/>
       <c r="J16" s="216" t="n"/>
       <c r="K16" s="216" t="n"/>
-      <c r="L16" s="217" t="n">
+      <c r="L16" s="276" t="n">
         <v>155704.27</v>
       </c>
       <c r="M16" s="216" t="n"/>
       <c r="N16" s="216" t="n"/>
       <c r="O16" s="216" t="n"/>
-      <c r="P16" s="217" t="n">
+      <c r="P16" s="276" t="n">
         <v>124563.41</v>
       </c>
-      <c r="Q16" s="217" t="n">
+      <c r="Q16" s="276" t="n">
         <v>186845.12</v>
       </c>
-      <c r="R16" s="217" t="n">
+      <c r="R16" s="276" t="n">
         <v>31140.85</v>
       </c>
       <c r="S16" s="216" t="n"/>
-      <c r="T16" s="218" t="n">
+      <c r="T16" s="277" t="n">
         <v>622817.0699999999</v>
       </c>
     </row>
@@ -20967,37 +22278,37 @@
           <t>Sistema UPS CA</t>
         </is>
       </c>
-      <c r="D17" s="215" t="n">
+      <c r="D17" s="275" t="n">
         <v>550434.3199999999</v>
       </c>
       <c r="E17" s="216" t="n"/>
-      <c r="F17" s="217" t="n">
+      <c r="F17" s="276" t="n">
         <v>55043.43</v>
       </c>
-      <c r="G17" s="217" t="n">
+      <c r="G17" s="276" t="n">
         <v>55043.43</v>
       </c>
       <c r="H17" s="216" t="n"/>
       <c r="I17" s="216" t="n"/>
       <c r="J17" s="216" t="n"/>
-      <c r="K17" s="217" t="n">
+      <c r="K17" s="276" t="n">
         <v>137608.58</v>
       </c>
-      <c r="L17" s="217" t="n">
+      <c r="L17" s="276" t="n">
         <v>110086.86</v>
       </c>
       <c r="M17" s="216" t="n"/>
       <c r="N17" s="216" t="n"/>
       <c r="O17" s="216" t="n"/>
       <c r="P17" s="216" t="n"/>
-      <c r="Q17" s="217" t="n">
+      <c r="Q17" s="276" t="n">
         <v>165130.3</v>
       </c>
-      <c r="R17" s="217" t="n">
+      <c r="R17" s="276" t="n">
         <v>27521.72</v>
       </c>
       <c r="S17" s="216" t="n"/>
-      <c r="T17" s="218" t="n">
+      <c r="T17" s="277" t="n">
         <v>550434.3199999999</v>
       </c>
     </row>
@@ -21018,37 +22329,37 @@
           <t>Sistema CC VCC</t>
         </is>
       </c>
-      <c r="D18" s="215" t="n">
+      <c r="D18" s="275" t="n">
         <v>274833.91</v>
       </c>
       <c r="E18" s="216" t="n"/>
-      <c r="F18" s="217" t="n">
+      <c r="F18" s="276" t="n">
         <v>27483.39</v>
       </c>
-      <c r="G18" s="217" t="n">
+      <c r="G18" s="276" t="n">
         <v>27483.39</v>
       </c>
       <c r="H18" s="216" t="n"/>
       <c r="I18" s="216" t="n"/>
       <c r="J18" s="216" t="n"/>
-      <c r="K18" s="217" t="n">
+      <c r="K18" s="276" t="n">
         <v>68708.48</v>
       </c>
-      <c r="L18" s="217" t="n">
+      <c r="L18" s="276" t="n">
         <v>54966.78</v>
       </c>
       <c r="M18" s="216" t="n"/>
       <c r="N18" s="216" t="n"/>
       <c r="O18" s="216" t="n"/>
       <c r="P18" s="216" t="n"/>
-      <c r="Q18" s="217" t="n">
+      <c r="Q18" s="276" t="n">
         <v>82450.17</v>
       </c>
-      <c r="R18" s="217" t="n">
+      <c r="R18" s="276" t="n">
         <v>13741.7</v>
       </c>
       <c r="S18" s="216" t="n"/>
-      <c r="T18" s="218" t="n">
+      <c r="T18" s="277" t="n">
         <v>274833.91</v>
       </c>
     </row>
@@ -21069,7 +22380,7 @@
           <t>CCM 380/220V lote 2</t>
         </is>
       </c>
-      <c r="D19" s="215" t="n">
+      <c r="D19" s="275" t="n">
         <v>451298.47</v>
       </c>
       <c r="E19" s="216" t="n"/>
@@ -21079,21 +22390,21 @@
       <c r="I19" s="216" t="n"/>
       <c r="J19" s="216" t="n"/>
       <c r="K19" s="216" t="n"/>
-      <c r="L19" s="217" t="n">
+      <c r="L19" s="276" t="n">
         <v>293344.01</v>
       </c>
       <c r="M19" s="216" t="n"/>
       <c r="N19" s="216" t="n"/>
       <c r="O19" s="216" t="n"/>
       <c r="P19" s="216" t="n"/>
-      <c r="Q19" s="217" t="n">
+      <c r="Q19" s="276" t="n">
         <v>135389.54</v>
       </c>
-      <c r="R19" s="217" t="n">
+      <c r="R19" s="276" t="n">
         <v>22564.92</v>
       </c>
       <c r="S19" s="216" t="n"/>
-      <c r="T19" s="218" t="n">
+      <c r="T19" s="277" t="n">
         <v>451298.47</v>
       </c>
     </row>
@@ -21114,7 +22425,7 @@
           <t>CCM 380/220V lote 2</t>
         </is>
       </c>
-      <c r="D20" s="215" t="n">
+      <c r="D20" s="275" t="n">
         <v>492942.64</v>
       </c>
       <c r="E20" s="216" t="n"/>
@@ -21124,21 +22435,21 @@
       <c r="I20" s="216" t="n"/>
       <c r="J20" s="216" t="n"/>
       <c r="K20" s="216" t="n"/>
-      <c r="L20" s="217" t="n">
+      <c r="L20" s="276" t="n">
         <v>320412.72</v>
       </c>
       <c r="M20" s="216" t="n"/>
       <c r="N20" s="216" t="n"/>
       <c r="O20" s="216" t="n"/>
       <c r="P20" s="216" t="n"/>
-      <c r="Q20" s="217" t="n">
+      <c r="Q20" s="276" t="n">
         <v>147882.79</v>
       </c>
-      <c r="R20" s="217" t="n">
+      <c r="R20" s="276" t="n">
         <v>24647.13</v>
       </c>
       <c r="S20" s="216" t="n"/>
-      <c r="T20" s="218" t="n">
+      <c r="T20" s="277" t="n">
         <v>492942.64</v>
       </c>
     </row>
@@ -21159,7 +22470,7 @@
           <t>CCM 380/220V lote 2</t>
         </is>
       </c>
-      <c r="D21" s="215" t="n">
+      <c r="D21" s="275" t="n">
         <v>552737.98</v>
       </c>
       <c r="E21" s="216" t="n"/>
@@ -21169,21 +22480,21 @@
       <c r="I21" s="216" t="n"/>
       <c r="J21" s="216" t="n"/>
       <c r="K21" s="216" t="n"/>
-      <c r="L21" s="217" t="n">
+      <c r="L21" s="276" t="n">
         <v>359279.69</v>
       </c>
       <c r="M21" s="216" t="n"/>
       <c r="N21" s="216" t="n"/>
       <c r="O21" s="216" t="n"/>
       <c r="P21" s="216" t="n"/>
-      <c r="Q21" s="217" t="n">
+      <c r="Q21" s="276" t="n">
         <v>165821.39</v>
       </c>
-      <c r="R21" s="217" t="n">
+      <c r="R21" s="276" t="n">
         <v>27636.9</v>
       </c>
       <c r="S21" s="216" t="n"/>
-      <c r="T21" s="218" t="n">
+      <c r="T21" s="277" t="n">
         <v>552737.9800000001</v>
       </c>
     </row>
@@ -21204,37 +22515,37 @@
           <t>Sala Eléctrica N°3 BT</t>
         </is>
       </c>
-      <c r="D22" s="215" t="n">
+      <c r="D22" s="275" t="n">
         <v>622817.0699999999</v>
       </c>
       <c r="E22" s="216" t="n"/>
       <c r="F22" s="216" t="n"/>
-      <c r="G22" s="217" t="n">
+      <c r="G22" s="276" t="n">
         <v>62281.71</v>
       </c>
-      <c r="H22" s="217" t="n">
+      <c r="H22" s="276" t="n">
         <v>62281.71</v>
       </c>
       <c r="I22" s="216" t="n"/>
       <c r="J22" s="216" t="n"/>
       <c r="K22" s="216" t="n"/>
-      <c r="L22" s="217" t="n">
+      <c r="L22" s="276" t="n">
         <v>155704.27</v>
       </c>
       <c r="M22" s="216" t="n"/>
       <c r="N22" s="216" t="n"/>
       <c r="O22" s="216" t="n"/>
-      <c r="P22" s="217" t="n">
+      <c r="P22" s="276" t="n">
         <v>124563.41</v>
       </c>
-      <c r="Q22" s="217" t="n">
+      <c r="Q22" s="276" t="n">
         <v>186845.12</v>
       </c>
-      <c r="R22" s="217" t="n">
+      <c r="R22" s="276" t="n">
         <v>31140.85</v>
       </c>
       <c r="S22" s="216" t="n"/>
-      <c r="T22" s="218" t="n">
+      <c r="T22" s="277" t="n">
         <v>622817.0699999999</v>
       </c>
     </row>
@@ -21255,37 +22566,37 @@
           <t>Sala Eléctrica N°3 BT</t>
         </is>
       </c>
-      <c r="D23" s="215" t="n">
+      <c r="D23" s="275" t="n">
         <v>622817.0699999999</v>
       </c>
       <c r="E23" s="216" t="n"/>
       <c r="F23" s="216" t="n"/>
-      <c r="G23" s="217" t="n">
+      <c r="G23" s="276" t="n">
         <v>62281.71</v>
       </c>
-      <c r="H23" s="217" t="n">
+      <c r="H23" s="276" t="n">
         <v>62281.71</v>
       </c>
       <c r="I23" s="216" t="n"/>
       <c r="J23" s="216" t="n"/>
       <c r="K23" s="216" t="n"/>
-      <c r="L23" s="217" t="n">
+      <c r="L23" s="276" t="n">
         <v>155704.27</v>
       </c>
       <c r="M23" s="216" t="n"/>
       <c r="N23" s="216" t="n"/>
       <c r="O23" s="216" t="n"/>
-      <c r="P23" s="217" t="n">
+      <c r="P23" s="276" t="n">
         <v>124563.41</v>
       </c>
-      <c r="Q23" s="217" t="n">
+      <c r="Q23" s="276" t="n">
         <v>186845.12</v>
       </c>
-      <c r="R23" s="217" t="n">
+      <c r="R23" s="276" t="n">
         <v>31140.85</v>
       </c>
       <c r="S23" s="216" t="n"/>
-      <c r="T23" s="218" t="n">
+      <c r="T23" s="277" t="n">
         <v>622817.0699999999</v>
       </c>
     </row>
@@ -21306,37 +22617,37 @@
           <t>Sala Eléctrica N°3 BT</t>
         </is>
       </c>
-      <c r="D24" s="215" t="n">
+      <c r="D24" s="275" t="n">
         <v>622817.0699999999</v>
       </c>
       <c r="E24" s="216" t="n"/>
       <c r="F24" s="216" t="n"/>
-      <c r="G24" s="217" t="n">
+      <c r="G24" s="276" t="n">
         <v>62281.71</v>
       </c>
-      <c r="H24" s="217" t="n">
+      <c r="H24" s="276" t="n">
         <v>62281.71</v>
       </c>
       <c r="I24" s="216" t="n"/>
       <c r="J24" s="216" t="n"/>
       <c r="K24" s="216" t="n"/>
-      <c r="L24" s="217" t="n">
+      <c r="L24" s="276" t="n">
         <v>155704.27</v>
       </c>
       <c r="M24" s="216" t="n"/>
       <c r="N24" s="216" t="n"/>
       <c r="O24" s="216" t="n"/>
-      <c r="P24" s="217" t="n">
+      <c r="P24" s="276" t="n">
         <v>124563.41</v>
       </c>
-      <c r="Q24" s="217" t="n">
+      <c r="Q24" s="276" t="n">
         <v>186845.12</v>
       </c>
-      <c r="R24" s="217" t="n">
+      <c r="R24" s="276" t="n">
         <v>31140.85</v>
       </c>
       <c r="S24" s="216" t="n"/>
-      <c r="T24" s="218" t="n">
+      <c r="T24" s="277" t="n">
         <v>622817.0699999999</v>
       </c>
     </row>
@@ -21357,37 +22668,37 @@
           <t>Sala Eléctrica N°3 BT</t>
         </is>
       </c>
-      <c r="D25" s="215" t="n">
+      <c r="D25" s="275" t="n">
         <v>622817.0699999999</v>
       </c>
       <c r="E25" s="216" t="n"/>
       <c r="F25" s="216" t="n"/>
-      <c r="G25" s="217" t="n">
+      <c r="G25" s="276" t="n">
         <v>62281.71</v>
       </c>
-      <c r="H25" s="217" t="n">
+      <c r="H25" s="276" t="n">
         <v>62281.71</v>
       </c>
       <c r="I25" s="216" t="n"/>
       <c r="J25" s="216" t="n"/>
       <c r="K25" s="216" t="n"/>
-      <c r="L25" s="217" t="n">
+      <c r="L25" s="276" t="n">
         <v>155704.27</v>
       </c>
       <c r="M25" s="216" t="n"/>
       <c r="N25" s="216" t="n"/>
       <c r="O25" s="216" t="n"/>
-      <c r="P25" s="217" t="n">
+      <c r="P25" s="276" t="n">
         <v>124563.41</v>
       </c>
-      <c r="Q25" s="217" t="n">
+      <c r="Q25" s="276" t="n">
         <v>186845.12</v>
       </c>
-      <c r="R25" s="217" t="n">
+      <c r="R25" s="276" t="n">
         <v>31140.85</v>
       </c>
       <c r="S25" s="216" t="n"/>
-      <c r="T25" s="218" t="n">
+      <c r="T25" s="277" t="n">
         <v>622817.0699999999</v>
       </c>
     </row>
@@ -21397,6 +22708,25 @@
           <t>OC S4 — 4508944973  |  Sala 4 MT  |  Total: USD 3,624,758</t>
         </is>
       </c>
+      <c r="B26" s="271" t="n"/>
+      <c r="C26" s="271" t="n"/>
+      <c r="D26" s="271" t="n"/>
+      <c r="E26" s="271" t="n"/>
+      <c r="F26" s="271" t="n"/>
+      <c r="G26" s="271" t="n"/>
+      <c r="H26" s="271" t="n"/>
+      <c r="I26" s="271" t="n"/>
+      <c r="J26" s="271" t="n"/>
+      <c r="K26" s="271" t="n"/>
+      <c r="L26" s="271" t="n"/>
+      <c r="M26" s="271" t="n"/>
+      <c r="N26" s="271" t="n"/>
+      <c r="O26" s="271" t="n"/>
+      <c r="P26" s="271" t="n"/>
+      <c r="Q26" s="271" t="n"/>
+      <c r="R26" s="271" t="n"/>
+      <c r="S26" s="271" t="n"/>
+      <c r="T26" s="272" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="220" t="inlineStr">
@@ -21415,37 +22745,37 @@
           <t>Tab. Distribución UPS SE#4</t>
         </is>
       </c>
-      <c r="D27" s="223" t="n">
+      <c r="D27" s="278" t="n">
         <v>25305.57</v>
       </c>
       <c r="E27" s="216" t="n"/>
-      <c r="F27" s="224" t="n">
+      <c r="F27" s="279" t="n">
         <v>2530.56</v>
       </c>
-      <c r="G27" s="224" t="n">
+      <c r="G27" s="279" t="n">
         <v>2530.56</v>
       </c>
       <c r="H27" s="216" t="n"/>
       <c r="I27" s="216" t="n"/>
       <c r="J27" s="216" t="n"/>
-      <c r="K27" s="224" t="n">
+      <c r="K27" s="279" t="n">
         <v>6326.39</v>
       </c>
-      <c r="L27" s="224" t="n">
+      <c r="L27" s="279" t="n">
         <v>5061.11</v>
       </c>
       <c r="M27" s="216" t="n"/>
       <c r="N27" s="216" t="n"/>
       <c r="O27" s="216" t="n"/>
-      <c r="P27" s="224" t="n">
+      <c r="P27" s="279" t="n">
         <v>7591.67</v>
       </c>
       <c r="Q27" s="216" t="n"/>
-      <c r="R27" s="224" t="n">
+      <c r="R27" s="279" t="n">
         <v>1265.28</v>
       </c>
       <c r="S27" s="216" t="n"/>
-      <c r="T27" s="218" t="n">
+      <c r="T27" s="277" t="n">
         <v>25305.57</v>
       </c>
     </row>
@@ -21466,37 +22796,37 @@
           <t>Tab. Distribución VCC SE#4</t>
         </is>
       </c>
-      <c r="D28" s="223" t="n">
+      <c r="D28" s="278" t="n">
         <v>29291.23</v>
       </c>
       <c r="E28" s="216" t="n"/>
-      <c r="F28" s="224" t="n">
+      <c r="F28" s="279" t="n">
         <v>2929.12</v>
       </c>
-      <c r="G28" s="224" t="n">
+      <c r="G28" s="279" t="n">
         <v>2929.12</v>
       </c>
       <c r="H28" s="216" t="n"/>
       <c r="I28" s="216" t="n"/>
       <c r="J28" s="216" t="n"/>
-      <c r="K28" s="224" t="n">
+      <c r="K28" s="279" t="n">
         <v>7322.81</v>
       </c>
-      <c r="L28" s="224" t="n">
+      <c r="L28" s="279" t="n">
         <v>5858.25</v>
       </c>
       <c r="M28" s="216" t="n"/>
       <c r="N28" s="216" t="n"/>
       <c r="O28" s="216" t="n"/>
-      <c r="P28" s="224" t="n">
+      <c r="P28" s="279" t="n">
         <v>8787.370000000001</v>
       </c>
       <c r="Q28" s="216" t="n"/>
-      <c r="R28" s="224" t="n">
+      <c r="R28" s="279" t="n">
         <v>1464.56</v>
       </c>
       <c r="S28" s="216" t="n"/>
-      <c r="T28" s="218" t="n">
+      <c r="T28" s="277" t="n">
         <v>29291.23</v>
       </c>
     </row>
@@ -21517,37 +22847,37 @@
           <t>Tab. Serv. Aux. SE#4</t>
         </is>
       </c>
-      <c r="D29" s="223" t="n">
+      <c r="D29" s="278" t="n">
         <v>66110.81</v>
       </c>
       <c r="E29" s="216" t="n"/>
-      <c r="F29" s="224" t="n">
+      <c r="F29" s="279" t="n">
         <v>6611.08</v>
       </c>
-      <c r="G29" s="224" t="n">
+      <c r="G29" s="279" t="n">
         <v>6611.08</v>
       </c>
       <c r="H29" s="216" t="n"/>
       <c r="I29" s="216" t="n"/>
       <c r="J29" s="216" t="n"/>
-      <c r="K29" s="224" t="n">
+      <c r="K29" s="279" t="n">
         <v>16527.7</v>
       </c>
-      <c r="L29" s="224" t="n">
+      <c r="L29" s="279" t="n">
         <v>13222.16</v>
       </c>
       <c r="M29" s="216" t="n"/>
       <c r="N29" s="216" t="n"/>
-      <c r="O29" s="224" t="n">
+      <c r="O29" s="279" t="n">
         <v>19833.24</v>
       </c>
       <c r="P29" s="216" t="n"/>
       <c r="Q29" s="216" t="n"/>
-      <c r="R29" s="224" t="n">
+      <c r="R29" s="279" t="n">
         <v>3305.54</v>
       </c>
       <c r="S29" s="216" t="n"/>
-      <c r="T29" s="218" t="n">
+      <c r="T29" s="277" t="n">
         <v>66110.8</v>
       </c>
     </row>
@@ -21568,33 +22898,33 @@
           <t>VFD MT Bombas</t>
         </is>
       </c>
-      <c r="D30" s="223" t="n">
+      <c r="D30" s="278" t="n">
         <v>396952.56</v>
       </c>
       <c r="E30" s="216" t="n"/>
       <c r="F30" s="216" t="n"/>
-      <c r="G30" s="224" t="n">
+      <c r="G30" s="279" t="n">
         <v>39695.26</v>
       </c>
       <c r="H30" s="216" t="n"/>
       <c r="I30" s="216" t="n"/>
       <c r="J30" s="216" t="n"/>
       <c r="K30" s="216" t="n"/>
-      <c r="L30" s="224" t="n">
+      <c r="L30" s="279" t="n">
         <v>218323.91</v>
       </c>
       <c r="M30" s="216" t="n"/>
       <c r="N30" s="216" t="n"/>
       <c r="O30" s="216" t="n"/>
-      <c r="P30" s="224" t="n">
+      <c r="P30" s="279" t="n">
         <v>119085.77</v>
       </c>
       <c r="Q30" s="216" t="n"/>
-      <c r="R30" s="224" t="n">
+      <c r="R30" s="279" t="n">
         <v>19847.63</v>
       </c>
       <c r="S30" s="216" t="n"/>
-      <c r="T30" s="218" t="n">
+      <c r="T30" s="277" t="n">
         <v>396952.57</v>
       </c>
     </row>
@@ -21615,37 +22945,37 @@
           <t>SWG MT 13.2/6.6kV Celdas</t>
         </is>
       </c>
-      <c r="D31" s="223" t="n">
+      <c r="D31" s="278" t="n">
         <v>517484.58</v>
       </c>
       <c r="E31" s="216" t="n"/>
-      <c r="F31" s="224" t="n">
+      <c r="F31" s="279" t="n">
         <v>51748.46</v>
       </c>
-      <c r="G31" s="224" t="n">
+      <c r="G31" s="279" t="n">
         <v>51748.46</v>
       </c>
       <c r="H31" s="216" t="n"/>
       <c r="I31" s="216" t="n"/>
       <c r="J31" s="216" t="n"/>
-      <c r="K31" s="224" t="n">
+      <c r="K31" s="279" t="n">
         <v>103496.92</v>
       </c>
-      <c r="L31" s="224" t="n">
+      <c r="L31" s="279" t="n">
         <v>129371.15</v>
       </c>
       <c r="M31" s="216" t="n"/>
       <c r="N31" s="216" t="n"/>
       <c r="O31" s="216" t="n"/>
-      <c r="P31" s="224" t="n">
+      <c r="P31" s="279" t="n">
         <v>155245.37</v>
       </c>
       <c r="Q31" s="216" t="n"/>
-      <c r="R31" s="224" t="n">
+      <c r="R31" s="279" t="n">
         <v>25874.23</v>
       </c>
       <c r="S31" s="216" t="n"/>
-      <c r="T31" s="218" t="n">
+      <c r="T31" s="277" t="n">
         <v>517484.59</v>
       </c>
     </row>
@@ -21666,37 +22996,37 @@
           <t>SWG MT Tableros lote 1</t>
         </is>
       </c>
-      <c r="D32" s="223" t="n">
+      <c r="D32" s="278" t="n">
         <v>386434.73</v>
       </c>
       <c r="E32" s="216" t="n"/>
-      <c r="F32" s="224" t="n">
+      <c r="F32" s="279" t="n">
         <v>38643.47</v>
       </c>
-      <c r="G32" s="224" t="n">
+      <c r="G32" s="279" t="n">
         <v>38643.47</v>
       </c>
       <c r="H32" s="216" t="n"/>
       <c r="I32" s="216" t="n"/>
       <c r="J32" s="216" t="n"/>
-      <c r="K32" s="224" t="n">
+      <c r="K32" s="279" t="n">
         <v>77286.95</v>
       </c>
-      <c r="L32" s="224" t="n">
+      <c r="L32" s="279" t="n">
         <v>96608.67999999999</v>
       </c>
       <c r="M32" s="216" t="n"/>
       <c r="N32" s="216" t="n"/>
       <c r="O32" s="216" t="n"/>
-      <c r="P32" s="224" t="n">
+      <c r="P32" s="279" t="n">
         <v>115930.42</v>
       </c>
       <c r="Q32" s="216" t="n"/>
-      <c r="R32" s="224" t="n">
+      <c r="R32" s="279" t="n">
         <v>19321.74</v>
       </c>
       <c r="S32" s="216" t="n"/>
-      <c r="T32" s="218" t="n">
+      <c r="T32" s="277" t="n">
         <v>386434.73</v>
       </c>
     </row>
@@ -21717,37 +23047,37 @@
           <t>Sala Eléctrica N°4 MT</t>
         </is>
       </c>
-      <c r="D33" s="223" t="n">
+      <c r="D33" s="278" t="n">
         <v>605581.3100000001</v>
       </c>
       <c r="E33" s="216" t="n"/>
-      <c r="F33" s="224" t="n">
+      <c r="F33" s="279" t="n">
         <v>60558.13</v>
       </c>
-      <c r="G33" s="224" t="n">
+      <c r="G33" s="279" t="n">
         <v>60558.13</v>
       </c>
       <c r="H33" s="216" t="n"/>
       <c r="I33" s="216" t="n"/>
       <c r="J33" s="216" t="n"/>
       <c r="K33" s="216" t="n"/>
-      <c r="L33" s="224" t="n">
+      <c r="L33" s="279" t="n">
         <v>151395.33</v>
       </c>
       <c r="M33" s="216" t="n"/>
       <c r="N33" s="216" t="n"/>
-      <c r="O33" s="224" t="n">
+      <c r="O33" s="279" t="n">
         <v>121116.26</v>
       </c>
-      <c r="P33" s="224" t="n">
+      <c r="P33" s="279" t="n">
         <v>181674.39</v>
       </c>
       <c r="Q33" s="216" t="n"/>
-      <c r="R33" s="224" t="n">
+      <c r="R33" s="279" t="n">
         <v>30279.07</v>
       </c>
       <c r="S33" s="216" t="n"/>
-      <c r="T33" s="218" t="n">
+      <c r="T33" s="277" t="n">
         <v>605581.3099999999</v>
       </c>
     </row>
@@ -21768,37 +23098,37 @@
           <t>SWG MT Tableros lote 2</t>
         </is>
       </c>
-      <c r="D34" s="223" t="n">
+      <c r="D34" s="278" t="n">
         <v>386434.73</v>
       </c>
       <c r="E34" s="216" t="n"/>
-      <c r="F34" s="224" t="n">
+      <c r="F34" s="279" t="n">
         <v>38643.47</v>
       </c>
-      <c r="G34" s="224" t="n">
+      <c r="G34" s="279" t="n">
         <v>38643.47</v>
       </c>
       <c r="H34" s="216" t="n"/>
       <c r="I34" s="216" t="n"/>
       <c r="J34" s="216" t="n"/>
-      <c r="K34" s="224" t="n">
+      <c r="K34" s="279" t="n">
         <v>77286.95</v>
       </c>
-      <c r="L34" s="224" t="n">
+      <c r="L34" s="279" t="n">
         <v>96608.67999999999</v>
       </c>
       <c r="M34" s="216" t="n"/>
       <c r="N34" s="216" t="n"/>
       <c r="O34" s="216" t="n"/>
-      <c r="P34" s="224" t="n">
+      <c r="P34" s="279" t="n">
         <v>115930.42</v>
       </c>
       <c r="Q34" s="216" t="n"/>
-      <c r="R34" s="224" t="n">
+      <c r="R34" s="279" t="n">
         <v>19321.74</v>
       </c>
       <c r="S34" s="216" t="n"/>
-      <c r="T34" s="218" t="n">
+      <c r="T34" s="277" t="n">
         <v>386434.73</v>
       </c>
     </row>
@@ -21819,37 +23149,37 @@
           <t>Sala Eléctrica N°4 MT</t>
         </is>
       </c>
-      <c r="D35" s="223" t="n">
+      <c r="D35" s="278" t="n">
         <v>605581.3100000001</v>
       </c>
       <c r="E35" s="216" t="n"/>
-      <c r="F35" s="224" t="n">
+      <c r="F35" s="279" t="n">
         <v>60558.13</v>
       </c>
-      <c r="G35" s="224" t="n">
+      <c r="G35" s="279" t="n">
         <v>60558.13</v>
       </c>
       <c r="H35" s="216" t="n"/>
       <c r="I35" s="216" t="n"/>
       <c r="J35" s="216" t="n"/>
       <c r="K35" s="216" t="n"/>
-      <c r="L35" s="224" t="n">
+      <c r="L35" s="279" t="n">
         <v>151395.33</v>
       </c>
       <c r="M35" s="216" t="n"/>
       <c r="N35" s="216" t="n"/>
-      <c r="O35" s="224" t="n">
+      <c r="O35" s="279" t="n">
         <v>121116.26</v>
       </c>
-      <c r="P35" s="224" t="n">
+      <c r="P35" s="279" t="n">
         <v>181674.39</v>
       </c>
       <c r="Q35" s="216" t="n"/>
-      <c r="R35" s="224" t="n">
+      <c r="R35" s="279" t="n">
         <v>30279.07</v>
       </c>
       <c r="S35" s="216" t="n"/>
-      <c r="T35" s="218" t="n">
+      <c r="T35" s="277" t="n">
         <v>605581.3099999999</v>
       </c>
     </row>
@@ -21870,37 +23200,37 @@
           <t>Sala Eléctrica N°4 MT</t>
         </is>
       </c>
-      <c r="D36" s="223" t="n">
+      <c r="D36" s="278" t="n">
         <v>605581.3100000001</v>
       </c>
       <c r="E36" s="216" t="n"/>
-      <c r="F36" s="224" t="n">
+      <c r="F36" s="279" t="n">
         <v>60558.13</v>
       </c>
-      <c r="G36" s="224" t="n">
+      <c r="G36" s="279" t="n">
         <v>60558.13</v>
       </c>
       <c r="H36" s="216" t="n"/>
       <c r="I36" s="216" t="n"/>
       <c r="J36" s="216" t="n"/>
       <c r="K36" s="216" t="n"/>
-      <c r="L36" s="224" t="n">
+      <c r="L36" s="279" t="n">
         <v>151395.33</v>
       </c>
       <c r="M36" s="216" t="n"/>
       <c r="N36" s="216" t="n"/>
-      <c r="O36" s="224" t="n">
+      <c r="O36" s="279" t="n">
         <v>121116.26</v>
       </c>
-      <c r="P36" s="224" t="n">
+      <c r="P36" s="279" t="n">
         <v>181674.39</v>
       </c>
       <c r="Q36" s="216" t="n"/>
-      <c r="R36" s="224" t="n">
+      <c r="R36" s="279" t="n">
         <v>30279.07</v>
       </c>
       <c r="S36" s="216" t="n"/>
-      <c r="T36" s="218" t="n">
+      <c r="T36" s="277" t="n">
         <v>605581.3099999999</v>
       </c>
     </row>
@@ -21910,43 +23240,45 @@
           <t>SUBTOTAL OC S3 — MENSUAL (USD)</t>
         </is>
       </c>
-      <c r="D38" s="226" t="n">
+      <c r="B38" s="271" t="n"/>
+      <c r="C38" s="272" t="n"/>
+      <c r="D38" s="280" t="n">
         <v>8027904</v>
       </c>
-      <c r="E38" s="226" t="n"/>
-      <c r="F38" s="226" t="n">
+      <c r="E38" s="280" t="n"/>
+      <c r="F38" s="280" t="n">
         <v>118668.15</v>
       </c>
-      <c r="G38" s="226" t="n">
+      <c r="G38" s="280" t="n">
         <v>503394.5900000001</v>
       </c>
-      <c r="H38" s="226" t="n">
+      <c r="H38" s="280" t="n">
         <v>360475.63</v>
       </c>
-      <c r="I38" s="226" t="n"/>
-      <c r="J38" s="226" t="n"/>
-      <c r="K38" s="226" t="n">
+      <c r="I38" s="280" t="n"/>
+      <c r="J38" s="280" t="n"/>
+      <c r="K38" s="280" t="n">
         <v>296670.38</v>
       </c>
-      <c r="L38" s="226" t="n">
+      <c r="L38" s="280" t="n">
         <v>3193444.12</v>
       </c>
-      <c r="M38" s="226" t="n"/>
-      <c r="N38" s="226" t="n">
+      <c r="M38" s="280" t="n"/>
+      <c r="N38" s="280" t="n">
         <v>122667.71</v>
       </c>
-      <c r="O38" s="226" t="n"/>
-      <c r="P38" s="226" t="n">
+      <c r="O38" s="280" t="n"/>
+      <c r="P38" s="280" t="n">
         <v>622817.05</v>
       </c>
-      <c r="Q38" s="226" t="n">
+      <c r="Q38" s="280" t="n">
         <v>2408371.180000001</v>
       </c>
-      <c r="R38" s="226" t="n">
+      <c r="R38" s="280" t="n">
         <v>401395.1899999999</v>
       </c>
-      <c r="S38" s="226" t="n"/>
-      <c r="T38" s="226" t="n">
+      <c r="S38" s="280" t="n"/>
+      <c r="T38" s="280" t="n">
         <v>8027904</v>
       </c>
     </row>
@@ -21956,39 +23288,41 @@
           <t>SUBTOTAL OC S4 — MENSUAL (USD)</t>
         </is>
       </c>
-      <c r="D39" s="228" t="n">
+      <c r="B39" s="271" t="n"/>
+      <c r="C39" s="272" t="n"/>
+      <c r="D39" s="281" t="n">
         <v>3624758.15</v>
       </c>
-      <c r="E39" s="228" t="n"/>
-      <c r="F39" s="228" t="n">
+      <c r="E39" s="281" t="n"/>
+      <c r="F39" s="281" t="n">
         <v>322780.55</v>
       </c>
-      <c r="G39" s="228" t="n">
+      <c r="G39" s="281" t="n">
         <v>362475.81</v>
       </c>
-      <c r="H39" s="228" t="n"/>
-      <c r="I39" s="228" t="n"/>
-      <c r="J39" s="228" t="n"/>
-      <c r="K39" s="228" t="n">
+      <c r="H39" s="281" t="n"/>
+      <c r="I39" s="281" t="n"/>
+      <c r="J39" s="281" t="n"/>
+      <c r="K39" s="281" t="n">
         <v>288247.72</v>
       </c>
-      <c r="L39" s="228" t="n">
+      <c r="L39" s="281" t="n">
         <v>1019239.93</v>
       </c>
-      <c r="M39" s="228" t="n"/>
-      <c r="N39" s="228" t="n"/>
-      <c r="O39" s="228" t="n">
+      <c r="M39" s="281" t="n"/>
+      <c r="N39" s="281" t="n"/>
+      <c r="O39" s="281" t="n">
         <v>383182.02</v>
       </c>
-      <c r="P39" s="228" t="n">
+      <c r="P39" s="281" t="n">
         <v>1067594.19</v>
       </c>
-      <c r="Q39" s="228" t="n"/>
-      <c r="R39" s="228" t="n">
+      <c r="Q39" s="281" t="n"/>
+      <c r="R39" s="281" t="n">
         <v>181237.93</v>
       </c>
-      <c r="S39" s="228" t="n"/>
-      <c r="T39" s="228" t="n">
+      <c r="S39" s="281" t="n"/>
+      <c r="T39" s="281" t="n">
         <v>3624758.15</v>
       </c>
     </row>
@@ -21998,45 +23332,47 @@
           <t>TOTAL COMBINADO S3+S4 — MENSUAL (USD)</t>
         </is>
       </c>
-      <c r="D40" s="230" t="n">
+      <c r="B40" s="271" t="n"/>
+      <c r="C40" s="272" t="n"/>
+      <c r="D40" s="282" t="n">
         <v>11652662.15</v>
       </c>
-      <c r="E40" s="230" t="n"/>
-      <c r="F40" s="230" t="n">
+      <c r="E40" s="282" t="n"/>
+      <c r="F40" s="282" t="n">
         <v>441448.7</v>
       </c>
-      <c r="G40" s="230" t="n">
+      <c r="G40" s="282" t="n">
         <v>865870.4000000001</v>
       </c>
-      <c r="H40" s="230" t="n">
+      <c r="H40" s="282" t="n">
         <v>360475.63</v>
       </c>
-      <c r="I40" s="230" t="n"/>
-      <c r="J40" s="230" t="n"/>
-      <c r="K40" s="230" t="n">
+      <c r="I40" s="282" t="n"/>
+      <c r="J40" s="282" t="n"/>
+      <c r="K40" s="282" t="n">
         <v>584918.1000000001</v>
       </c>
-      <c r="L40" s="230" t="n">
+      <c r="L40" s="282" t="n">
         <v>4212684.05</v>
       </c>
-      <c r="M40" s="230" t="n"/>
-      <c r="N40" s="230" t="n">
+      <c r="M40" s="282" t="n"/>
+      <c r="N40" s="282" t="n">
         <v>122667.71</v>
       </c>
-      <c r="O40" s="230" t="n">
+      <c r="O40" s="282" t="n">
         <v>383182.02</v>
       </c>
-      <c r="P40" s="230" t="n">
+      <c r="P40" s="282" t="n">
         <v>1690411.24</v>
       </c>
-      <c r="Q40" s="230" t="n">
+      <c r="Q40" s="282" t="n">
         <v>2408371.180000001</v>
       </c>
-      <c r="R40" s="230" t="n">
+      <c r="R40" s="282" t="n">
         <v>582633.12</v>
       </c>
-      <c r="S40" s="230" t="n"/>
-      <c r="T40" s="230" t="n">
+      <c r="S40" s="282" t="n"/>
+      <c r="T40" s="282" t="n">
         <v>11652662.15</v>
       </c>
     </row>
@@ -22046,53 +23382,55 @@
           <t>ACUMULADO (Curva S) — USD</t>
         </is>
       </c>
+      <c r="B41" s="271" t="n"/>
+      <c r="C41" s="272" t="n"/>
       <c r="D41" s="232" t="inlineStr"/>
-      <c r="E41" s="233" t="n">
+      <c r="E41" s="283" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="233" t="n">
+      <c r="F41" s="283" t="n">
         <v>441448.7</v>
       </c>
-      <c r="G41" s="233" t="n">
+      <c r="G41" s="283" t="n">
         <v>1307319.1</v>
       </c>
-      <c r="H41" s="233" t="n">
+      <c r="H41" s="283" t="n">
         <v>1667794.73</v>
       </c>
-      <c r="I41" s="233" t="n">
+      <c r="I41" s="283" t="n">
         <v>1667794.73</v>
       </c>
-      <c r="J41" s="233" t="n">
+      <c r="J41" s="283" t="n">
         <v>1667794.73</v>
       </c>
-      <c r="K41" s="233" t="n">
+      <c r="K41" s="283" t="n">
         <v>2252712.83</v>
       </c>
-      <c r="L41" s="233" t="n">
+      <c r="L41" s="283" t="n">
         <v>6465396.88</v>
       </c>
-      <c r="M41" s="233" t="n">
+      <c r="M41" s="283" t="n">
         <v>6465396.88</v>
       </c>
-      <c r="N41" s="233" t="n">
+      <c r="N41" s="283" t="n">
         <v>6588064.59</v>
       </c>
-      <c r="O41" s="233" t="n">
+      <c r="O41" s="283" t="n">
         <v>6971246.609999999</v>
       </c>
-      <c r="P41" s="233" t="n">
+      <c r="P41" s="283" t="n">
         <v>8661657.85</v>
       </c>
-      <c r="Q41" s="233" t="n">
+      <c r="Q41" s="283" t="n">
         <v>11070029.03</v>
       </c>
-      <c r="R41" s="233" t="n">
+      <c r="R41" s="283" t="n">
         <v>11652662.15</v>
       </c>
-      <c r="S41" s="233" t="n">
+      <c r="S41" s="283" t="n">
         <v>11652662.15</v>
       </c>
-      <c r="T41" s="233" t="n">
+      <c r="T41" s="283" t="n">
         <v>11652662.15</v>
       </c>
     </row>

</xml_diff>